<commit_message>
lista de chequeo def
</commit_message>
<xml_diff>
--- a/Lista de chequeo.xlsx
+++ b/Lista de chequeo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENA\Downloads\CDL-Proyecto-6to-trimestre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB62382-91C6-491A-A20E-E956DBB94056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A762D419-95A7-49DD-92AD-982036A16A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="47">
   <si>
     <t>Lista de Chequeo</t>
   </si>
@@ -172,9 +172,6 @@
   </si>
   <si>
     <t>En el proyecto se evidencia que el front end web consuma la API REST (Angular, Vue.js, react u otros), con un avance del 80% de la codificación</t>
-  </si>
-  <si>
-    <t>En el proyecto se evidencia el uso de sistemas de control de versiones.B29:E31+30:30</t>
   </si>
 </sst>
 </file>
@@ -523,24 +520,6 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <u val="none"/>
@@ -692,6 +671,22 @@
       </border>
     </dxf>
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <bottom style="thin">
           <color indexed="64"/>
@@ -706,12 +701,14 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
   </dxfs>
@@ -728,13 +725,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="B2:E40" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="B2:E40" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="B2:E40" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Trimestre" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Lista de Chequeo" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Entregables" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="NOTAS" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Trimestre" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Lista de Chequeo" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Entregables" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="NOTAS" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1362,9 +1359,7 @@
       <c r="E29" s="15"/>
     </row>
     <row r="30" spans="1:9" ht="45.75">
-      <c r="A30" s="23" t="s">
-        <v>47</v>
-      </c>
+      <c r="A30" s="23"/>
       <c r="B30" s="12" t="s">
         <v>33</v>
       </c>

</xml_diff>